<commit_message>
feat(PDG-65): add SEC_PH_ADVISORIES media source
SEC advisories via Cloudflare bypass with the PDF as the record file, stop_after_known discovery, and author/language/categories from the page metadata. mediaPickLists.xlsx also carries the DTI_PH SourceName row (binary file, cannot be split).
</commit_message>
<xml_diff>
--- a/data/rules/mediaPickLists.xlsx
+++ b/data/rules/mediaPickLists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CC95F0-89EA-48AB-8EE8-BF21788EDBDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD780126-448F-4AF6-8F9F-D9A2942F40E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="73">
   <si>
     <t>Path</t>
   </si>
@@ -233,6 +233,12 @@
   </si>
   <si>
     <t>DTI_PH</t>
+  </si>
+  <si>
+    <t>SEC_PH_ADVISORIES</t>
+  </si>
+  <si>
+    <t>SEC_PH</t>
   </si>
 </sst>
 </file>
@@ -802,34 +808,40 @@
       <c r="B12" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="C12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
-        <v>55</v>
-      </c>
+      <c r="D13" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -837,12 +849,12 @@
         <v>53</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -850,12 +862,12 @@
         <v>53</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -863,88 +875,86 @@
         <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>70</v>
+      <c r="B18" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
+      <c r="E18" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="19" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>16</v>
+        <v>53</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>70</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="6" t="s">
-        <v>17</v>
-      </c>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="E20" s="6"/>
     </row>
     <row r="21" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -952,12 +962,12 @@
         <v>22</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -965,49 +975,49 @@
         <v>22</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
+      <c r="E25" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="26" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
-      <c r="E27" s="6" t="s">
-        <v>32</v>
-      </c>
+      <c r="E27" s="6"/>
     </row>
     <row r="28" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1036,12 +1046,12 @@
         <v>8</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1049,12 +1059,12 @@
         <v>8</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1062,40 +1072,52 @@
         <v>8</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
+      <c r="A33" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
+      <c r="E33" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="34" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
+      <c r="E34" s="6" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="35" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="6"/>

</xml_diff>

<commit_message>
feat(PDG-78): recategorize media datasets as Regulatory or Media
</commit_message>
<xml_diff>
--- a/data/rules/mediaPickLists.xlsx
+++ b/data/rules/mediaPickLists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD222CA-AEA2-4B06-A72C-D877727DCB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C6FDB6-3753-4328-8A0B-B70CD1F6DFCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="78">
   <si>
     <t>Path</t>
   </si>
@@ -55,13 +55,7 @@
     <t>Identifiers.Type</t>
   </si>
   <si>
-    <t>Press Release</t>
-  </si>
-  <si>
     <t>Official statement or press release issued by a government agency, regulator, company, or organization.</t>
-  </si>
-  <si>
-    <t>News Article</t>
   </si>
   <si>
     <t>News report published by a media outlet or news organization.</t>
@@ -239,6 +233,27 @@
   </si>
   <si>
     <t>SEC_PH</t>
+  </si>
+  <si>
+    <t>Regulatory</t>
+  </si>
+  <si>
+    <t>DTI_PH_FAIR_TRADE_UPDATES</t>
+  </si>
+  <si>
+    <t>ADB_CASE_SUMMARIES</t>
+  </si>
+  <si>
+    <t>ADB</t>
+  </si>
+  <si>
+    <t>Asian Development Bank.</t>
+  </si>
+  <si>
+    <t>Thumbnail</t>
+  </si>
+  <si>
+    <t>Main image shown with the article on listing pages.</t>
   </si>
 </sst>
 </file>
@@ -659,7 +674,7 @@
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -667,12 +682,12 @@
         <v>5</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
       <c r="E3" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -680,12 +695,12 @@
         <v>7</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -693,331 +708,337 @@
         <v>7</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
       <c r="E5" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="D10" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E11" s="6"/>
     </row>
     <row r="12" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>72</v>
+        <v>51</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="6" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6" t="s">
-        <v>55</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6" t="s">
-        <v>57</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>70</v>
+        <v>51</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>58</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
+      <c r="E19" s="6" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="20" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
+      <c r="E20" s="6" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="21" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>16</v>
+        <v>51</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
-      <c r="E21" s="6" t="s">
-        <v>17</v>
-      </c>
+      <c r="E21" s="6"/>
     </row>
     <row r="22" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="E22" s="6"/>
     </row>
     <row r="23" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
+      <c r="E27" s="6" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="28" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1043,41 +1064,39 @@
     </row>
     <row r="29" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="6" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="6" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
-      <c r="E30" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="E30" s="6"/>
     </row>
     <row r="31" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1085,12 +1104,12 @@
         <v>8</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -1098,54 +1117,78 @@
         <v>8</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="6"/>
-      <c r="B35" s="6"/>
+      <c r="A35" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>34</v>
+      </c>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
+      <c r="E35" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="36" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="6"/>
-      <c r="B36" s="6"/>
+      <c r="A36" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
+      <c r="E36" s="6" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="37" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="6"/>
-      <c r="B37" s="6"/>
+      <c r="A37" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>76</v>
+      </c>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
+      <c r="E37" s="6" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="38" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="6"/>
-      <c r="B38" s="6"/>
+      <c r="A38" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
+      <c r="E38" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="39" spans="1:26" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="6"/>

</xml_diff>